<commit_message>
GASCDS-1081: process excel file
</commit_message>
<xml_diff>
--- a/ni_api/core.Tests/TestData/test_ni_list.xlsx
+++ b/ni_api/core.Tests/TestData/test_ni_list.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="1 - Active Locations" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="59">
   <si>
     <t xml:space="preserve">Location ID</t>
   </si>
@@ -172,6 +172,12 @@
   </si>
   <si>
     <t xml:space="preserve">test@testing.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1-10000302983</t>
+  </si>
+  <si>
+    <t xml:space="preserve">My Other Organisation</t>
   </si>
   <si>
     <t xml:space="preserve">Nominated Individual</t>
@@ -296,32 +302,36 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -652,7 +662,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="74.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="21.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="21.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="16.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="8"/>
@@ -741,16 +751,16 @@
     </row>
     <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>41</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>46054</v>
@@ -759,22 +769,22 @@
         <v>43</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="J3" s="3" t="s">
         <v>47</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -800,8 +810,8 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
-        <v>56</v>
+      <c r="A1" s="7" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>